<commit_message>
Drive stats and last-updated date from Google Sheets
- Stats card row now reads from Total tab (Label, Total columns)
  Last row gets the red highlight (hardcoded), keeping the design
- Footer 'Dernière mise à jour' reads from Update_date tab
  (Key=Last_updated, Value=...)
- Both feeds are optional: missing env vars hide their blocks
- Add VITE_STATS_CSV_URL and VITE_META_CSV_URL to deploy workflow
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Timeline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Stats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Meta" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -861,4 +863,112 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Personnes à bord</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Nationalités</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Décès</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Last_updated</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>6 mai 2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>